<commit_message>
docs(tabs): add Allocation type to Survey_Structure_Template.xlsx
- Variable Type Reference sheet: new Allocation row after Open_End —
  description, Columns (>1), key features, and example
- Questions sheet: Columns field description updated to mention Allocation
  alongside Multi_Mention and Ranking

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Survey_Structure_Template.xlsx
+++ b/modules/tabs/templates/Survey_Structure_Template.xlsx
@@ -1,30 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duncan/Dev/Turas/modules/tabs/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E5E558-94E6-F14C-8A7C-12FD144E361A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="36040" windowHeight="19140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="36040" windowHeight="19140" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Project" sheetId="1" r:id="rId1"/>
-    <sheet name="Questions" sheetId="2" r:id="rId2"/>
-    <sheet name="Options" sheetId="3" r:id="rId3"/>
-    <sheet name="Composite_Metrics" sheetId="4" r:id="rId4"/>
-    <sheet name="Variable Type Reference" sheetId="5" r:id="rId5"/>
+    <sheet name="Project" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Options" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Composite_Metrics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Variable Type Reference" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="239">
   <si>
     <t>TURAS Survey Structure - Project Setup</t>
   </si>
@@ -68,7 +61,7 @@
     <t>project_name</t>
   </si>
   <si>
-    <t/>
+    <t>NA</t>
   </si>
   <si>
     <t>REQUIRED</t>
@@ -753,12 +746,31 @@
       <t>Only for Likert Questions</t>
     </r>
   </si>
+  <si>
+    <t xml:space="preserve">Allocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constant-sum / budget allocation. One numeric column per option ({code}_1 ... {code}_N). Reports mean allocation per option, cross-tabbed by banner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;1 (# options)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean per option cross-tabbed by banner. Zeros retained. Optional significance tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand spend share, budget distribution, 100-point allocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Number of data columns: 1 for most types; &gt;1 for Multi_Mention (# options), Ranking (# items), and Allocation (# options).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -767,91 +779,76 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF323367"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF546E7A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <b/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF323367"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FFD32F2F"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <b/>
     </font>
     <font>
-      <i/>
       <sz val="9"/>
       <color rgb="FF546E7A"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <i/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF546E7A"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF388E3C"/>
       <name val="Calibri"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF323367"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF546E7A"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF323367"/>
+      <name val="Calibri"/>
+      <b/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF37474F"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF546E7A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -888,12 +885,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8EAF6"/>
+        <fgColor rgb="FFF8F9FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
+        <fgColor rgb="FFE8EAF6"/>
       </patternFill>
     </fill>
     <fill>
@@ -923,7 +920,6 @@
       <bottom style="thin">
         <color rgb="FFB0BEC5"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -938,7 +934,6 @@
       <bottom style="thin">
         <color rgb="FF323367"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -946,54 +941,54 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1290,59 +1285,37 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{B2840D3F-692D-9B4D-B71B-63668B586799}">
-  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;b74a9558-bf5e-45da-af0a-d3db6bbbaa48&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="38.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="55.6640625" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" customWidth="1"/>
+    <col min="1" max="1" width="38.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="55.6640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+    </row>
+    <row r="3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1359,7 +1332,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -1376,16 +1349,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+    <row r="6">
+      <c r="A6" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+    </row>
+    <row r="7">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
@@ -1402,7 +1375,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" s="7" t="s">
         <v>18</v>
       </c>
@@ -1419,7 +1392,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" s="7" t="s">
         <v>21</v>
       </c>
@@ -1436,7 +1409,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" s="7" t="s">
         <v>24</v>
       </c>
@@ -1453,7 +1426,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" s="7" t="s">
         <v>28</v>
       </c>
@@ -1470,7 +1443,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" s="12" t="s">
         <v>31</v>
       </c>
@@ -1487,7 +1460,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" s="12" t="s">
         <v>33</v>
       </c>
@@ -1504,16 +1477,16 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="18" t="s">
+    <row r="14">
+      <c r="A14" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+    </row>
+    <row r="15">
       <c r="A15" s="7" t="s">
         <v>36</v>
       </c>
@@ -1530,7 +1503,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16" s="7" t="s">
         <v>39</v>
       </c>
@@ -1547,7 +1520,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17" s="7" t="s">
         <v>43</v>
       </c>
@@ -1564,16 +1537,16 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="18" t="s">
+    <row r="18">
+      <c r="A18" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+    </row>
+    <row r="19">
       <c r="A19" s="12" t="s">
         <v>47</v>
       </c>
@@ -1590,7 +1563,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="26" x14ac:dyDescent="0.2">
+    <row r="20" ht="26" customHeight="1">
       <c r="A20" s="12" t="s">
         <v>51</v>
       </c>
@@ -1607,7 +1580,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" s="12" t="s">
         <v>54</v>
       </c>
@@ -1624,7 +1597,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" s="12" t="s">
         <v>57</v>
       </c>
@@ -1663,52 +1636,54 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K62"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="45.6640625" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="8" width="18.6640625" customWidth="1"/>
-    <col min="9" max="10" width="12.6640625" customWidth="1"/>
-    <col min="11" max="11" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="45.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="30.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-    </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
         <v>62</v>
       </c>
@@ -1743,7 +1718,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="45" customHeight="1">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1754,7 +1729,7 @@
         <v>75</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>76</v>
+        <v>239</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>77</v>
@@ -1778,287 +1753,287 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5">
+      <c r="A5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="F5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="14" t="s">
+      <c r="F5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="18" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+    <row r="6">
+      <c r="A6" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="F6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="14" t="s">
+      <c r="F6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="18" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+    <row r="7">
+      <c r="A7" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="14" t="s">
+      <c r="F7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="18" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
+    <row r="8">
+      <c r="A8" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="F8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="14" t="s">
+      <c r="F8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="18" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+    <row r="9">
+      <c r="A9" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="14" t="s">
+      <c r="F9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="18" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+    <row r="10">
+      <c r="A10" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="I10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K10" s="14" t="s">
+      <c r="I10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="18" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
+    <row r="11">
+      <c r="A11" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="F11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="14">
+      <c r="F11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="J11" s="14">
+      <c r="J11" s="18" t="n">
         <v>99</v>
       </c>
-      <c r="K11" s="14" t="s">
+      <c r="K11" s="18" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+    <row r="12">
+      <c r="A12" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K12" s="14" t="s">
+      <c r="F12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="18" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -2071,7 +2046,7 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -2084,7 +2059,7 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -2097,7 +2072,7 @@
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -2110,7 +2085,7 @@
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -2123,7 +2098,7 @@
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -2136,7 +2111,7 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -2149,7 +2124,7 @@
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -2162,7 +2137,7 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -2175,7 +2150,7 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -2188,7 +2163,7 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -2201,7 +2176,7 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -2214,7 +2189,7 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -2227,7 +2202,7 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -2240,7 +2215,7 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2253,7 +2228,7 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -2266,7 +2241,7 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -2279,7 +2254,7 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -2292,7 +2267,7 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31">
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -2305,7 +2280,7 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -2318,7 +2293,7 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -2331,7 +2306,7 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2344,7 +2319,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -2357,7 +2332,7 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -2370,7 +2345,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -2383,7 +2358,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -2396,7 +2371,7 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -2409,7 +2384,7 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -2422,7 +2397,7 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -2435,7 +2410,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -2448,7 +2423,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -2461,7 +2436,7 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -2474,7 +2449,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -2487,7 +2462,7 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -2500,7 +2475,7 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -2513,7 +2488,7 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -2526,7 +2501,7 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -2539,7 +2514,7 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -2552,7 +2527,7 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51">
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -2565,7 +2540,7 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52">
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -2578,7 +2553,7 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53">
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -2591,7 +2566,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54">
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -2604,7 +2579,7 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -2617,7 +2592,7 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -2630,7 +2605,7 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57">
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -2643,7 +2618,7 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58">
       <c r="A58" s="8"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8"/>
@@ -2656,7 +2631,7 @@
       <c r="J58" s="8"/>
       <c r="K58" s="8"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59">
       <c r="A59" s="8"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8"/>
@@ -2669,7 +2644,7 @@
       <c r="J59" s="8"/>
       <c r="K59" s="8"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60">
       <c r="A60" s="8"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -2682,7 +2657,7 @@
       <c r="J60" s="8"/>
       <c r="K60" s="8"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61">
       <c r="A61" s="8"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -2695,7 +2670,7 @@
       <c r="J61" s="8"/>
       <c r="K61" s="8"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62">
       <c r="A62" s="8"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -2738,51 +2713,54 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K221"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="25.6640625" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" customWidth="1"/>
-    <col min="4" max="5" width="14.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="7" max="8" width="14.6640625" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" customWidth="1"/>
-    <col min="10" max="11" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="30.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-    </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
         <v>62</v>
       </c>
@@ -2817,7 +2795,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="97" customHeight="1">
       <c r="A4" s="10" t="s">
         <v>136</v>
       </c>
@@ -2852,602 +2830,602 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5">
+      <c r="A5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="F5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+      <c r="F6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
+      <c r="F7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="F8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="F9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="14">
+      <c r="F10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="14" t="s">
+      <c r="H10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K10" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
+      <c r="J10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="14">
+      <c r="F11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="14" t="s">
+      <c r="H11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="J11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K11" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+      <c r="J11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="14">
+      <c r="F12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K12" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="H12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F13" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13" s="14">
+      <c r="F13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H13" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I13" s="14" t="s">
+      <c r="H13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="J13" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K13" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
+      <c r="J13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F14" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G14" s="14">
+      <c r="F14" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I14" s="14" t="s">
+      <c r="H14" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="J14" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K14" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
+      <c r="J14" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" s="14">
+      <c r="F15" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="18" t="n">
         <v>-100</v>
       </c>
-      <c r="H15" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="14" t="s">
+      <c r="H15" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="J15" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K15" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+      <c r="J15" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="14">
+      <c r="F16" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="18" t="n">
         <v>-50</v>
       </c>
-      <c r="H16" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I16" s="14" t="s">
+      <c r="H16" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="J16" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="J16" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E17" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F17" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" s="14">
+      <c r="F17" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J17" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K17" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="H17" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" s="14">
+      <c r="F18" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="H18" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I18" s="14" t="s">
+      <c r="H18" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="J18" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K18" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="J18" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F19" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G19" s="14">
+      <c r="F19" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H19" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I19" s="14" t="s">
+      <c r="H19" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="J19" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K19" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
+      <c r="J19" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F20" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J20" s="14">
+      <c r="F20" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="K20" s="14">
+      <c r="K20" s="18" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
+    <row r="21">
+      <c r="A21" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="F21" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J21" s="14">
+      <c r="F21" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="K21" s="14">
+      <c r="K21" s="18" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -3460,7 +3438,7 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -3473,7 +3451,7 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -3486,7 +3464,7 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -3499,7 +3477,7 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -3512,7 +3490,7 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -3525,7 +3503,7 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -3538,7 +3516,7 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -3551,7 +3529,7 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -3564,7 +3542,7 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31">
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -3577,7 +3555,7 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -3590,7 +3568,7 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -3603,7 +3581,7 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -3616,7 +3594,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -3629,7 +3607,7 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -3642,7 +3620,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -3655,7 +3633,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -3668,7 +3646,7 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -3681,7 +3659,7 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -3694,7 +3672,7 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -3707,7 +3685,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -3720,7 +3698,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -3733,7 +3711,7 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -3746,7 +3724,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -3759,7 +3737,7 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -3772,7 +3750,7 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -3785,7 +3763,7 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -3798,7 +3776,7 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -3811,7 +3789,7 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -3824,7 +3802,7 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51">
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -3837,7 +3815,7 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52">
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -3850,7 +3828,7 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53">
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -3863,7 +3841,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54">
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -3876,7 +3854,7 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -3889,7 +3867,7 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -3902,7 +3880,7 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57">
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -3915,7 +3893,7 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58">
       <c r="A58" s="8"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8"/>
@@ -3928,7 +3906,7 @@
       <c r="J58" s="8"/>
       <c r="K58" s="8"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59">
       <c r="A59" s="8"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8"/>
@@ -3941,7 +3919,7 @@
       <c r="J59" s="8"/>
       <c r="K59" s="8"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60">
       <c r="A60" s="8"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -3954,7 +3932,7 @@
       <c r="J60" s="8"/>
       <c r="K60" s="8"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61">
       <c r="A61" s="8"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -3967,7 +3945,7 @@
       <c r="J61" s="8"/>
       <c r="K61" s="8"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62">
       <c r="A62" s="8"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -3980,7 +3958,7 @@
       <c r="J62" s="8"/>
       <c r="K62" s="8"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63">
       <c r="A63" s="8"/>
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
@@ -3993,7 +3971,7 @@
       <c r="J63" s="8"/>
       <c r="K63" s="8"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="64">
       <c r="A64" s="8"/>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -4006,7 +3984,7 @@
       <c r="J64" s="8"/>
       <c r="K64" s="8"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65">
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
@@ -4019,7 +3997,7 @@
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="66">
       <c r="A66" s="8"/>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -4032,7 +4010,7 @@
       <c r="J66" s="8"/>
       <c r="K66" s="8"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="67">
       <c r="A67" s="8"/>
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
@@ -4045,7 +4023,7 @@
       <c r="J67" s="8"/>
       <c r="K67" s="8"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="68">
       <c r="A68" s="8"/>
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
@@ -4058,7 +4036,7 @@
       <c r="J68" s="8"/>
       <c r="K68" s="8"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="69">
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
@@ -4071,7 +4049,7 @@
       <c r="J69" s="8"/>
       <c r="K69" s="8"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="70">
       <c r="A70" s="8"/>
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
@@ -4084,7 +4062,7 @@
       <c r="J70" s="8"/>
       <c r="K70" s="8"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="71">
       <c r="A71" s="8"/>
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
@@ -4097,7 +4075,7 @@
       <c r="J71" s="8"/>
       <c r="K71" s="8"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="72">
       <c r="A72" s="8"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
@@ -4110,7 +4088,7 @@
       <c r="J72" s="8"/>
       <c r="K72" s="8"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="73">
       <c r="A73" s="8"/>
       <c r="B73" s="8"/>
       <c r="C73" s="8"/>
@@ -4123,7 +4101,7 @@
       <c r="J73" s="8"/>
       <c r="K73" s="8"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="74">
       <c r="A74" s="8"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8"/>
@@ -4136,7 +4114,7 @@
       <c r="J74" s="8"/>
       <c r="K74" s="8"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="75">
       <c r="A75" s="8"/>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -4149,7 +4127,7 @@
       <c r="J75" s="8"/>
       <c r="K75" s="8"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="76">
       <c r="A76" s="8"/>
       <c r="B76" s="8"/>
       <c r="C76" s="8"/>
@@ -4162,7 +4140,7 @@
       <c r="J76" s="8"/>
       <c r="K76" s="8"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="77">
       <c r="A77" s="8"/>
       <c r="B77" s="8"/>
       <c r="C77" s="8"/>
@@ -4175,7 +4153,7 @@
       <c r="J77" s="8"/>
       <c r="K77" s="8"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="78">
       <c r="A78" s="8"/>
       <c r="B78" s="8"/>
       <c r="C78" s="8"/>
@@ -4188,7 +4166,7 @@
       <c r="J78" s="8"/>
       <c r="K78" s="8"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="79">
       <c r="A79" s="8"/>
       <c r="B79" s="8"/>
       <c r="C79" s="8"/>
@@ -4201,7 +4179,7 @@
       <c r="J79" s="8"/>
       <c r="K79" s="8"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="80">
       <c r="A80" s="8"/>
       <c r="B80" s="8"/>
       <c r="C80" s="8"/>
@@ -4214,7 +4192,7 @@
       <c r="J80" s="8"/>
       <c r="K80" s="8"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="81">
       <c r="A81" s="8"/>
       <c r="B81" s="8"/>
       <c r="C81" s="8"/>
@@ -4227,7 +4205,7 @@
       <c r="J81" s="8"/>
       <c r="K81" s="8"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="82">
       <c r="A82" s="8"/>
       <c r="B82" s="8"/>
       <c r="C82" s="8"/>
@@ -4240,7 +4218,7 @@
       <c r="J82" s="8"/>
       <c r="K82" s="8"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="83">
       <c r="A83" s="8"/>
       <c r="B83" s="8"/>
       <c r="C83" s="8"/>
@@ -4253,7 +4231,7 @@
       <c r="J83" s="8"/>
       <c r="K83" s="8"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="84">
       <c r="A84" s="8"/>
       <c r="B84" s="8"/>
       <c r="C84" s="8"/>
@@ -4266,7 +4244,7 @@
       <c r="J84" s="8"/>
       <c r="K84" s="8"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="85">
       <c r="A85" s="8"/>
       <c r="B85" s="8"/>
       <c r="C85" s="8"/>
@@ -4279,7 +4257,7 @@
       <c r="J85" s="8"/>
       <c r="K85" s="8"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="86">
       <c r="A86" s="8"/>
       <c r="B86" s="8"/>
       <c r="C86" s="8"/>
@@ -4292,7 +4270,7 @@
       <c r="J86" s="8"/>
       <c r="K86" s="8"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="87">
       <c r="A87" s="8"/>
       <c r="B87" s="8"/>
       <c r="C87" s="8"/>
@@ -4305,7 +4283,7 @@
       <c r="J87" s="8"/>
       <c r="K87" s="8"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="88">
       <c r="A88" s="8"/>
       <c r="B88" s="8"/>
       <c r="C88" s="8"/>
@@ -4318,7 +4296,7 @@
       <c r="J88" s="8"/>
       <c r="K88" s="8"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="89">
       <c r="A89" s="8"/>
       <c r="B89" s="8"/>
       <c r="C89" s="8"/>
@@ -4331,7 +4309,7 @@
       <c r="J89" s="8"/>
       <c r="K89" s="8"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="90">
       <c r="A90" s="8"/>
       <c r="B90" s="8"/>
       <c r="C90" s="8"/>
@@ -4344,7 +4322,7 @@
       <c r="J90" s="8"/>
       <c r="K90" s="8"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="91">
       <c r="A91" s="8"/>
       <c r="B91" s="8"/>
       <c r="C91" s="8"/>
@@ -4357,7 +4335,7 @@
       <c r="J91" s="8"/>
       <c r="K91" s="8"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="92">
       <c r="A92" s="8"/>
       <c r="B92" s="8"/>
       <c r="C92" s="8"/>
@@ -4370,7 +4348,7 @@
       <c r="J92" s="8"/>
       <c r="K92" s="8"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="93">
       <c r="A93" s="8"/>
       <c r="B93" s="8"/>
       <c r="C93" s="8"/>
@@ -4383,7 +4361,7 @@
       <c r="J93" s="8"/>
       <c r="K93" s="8"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="94">
       <c r="A94" s="8"/>
       <c r="B94" s="8"/>
       <c r="C94" s="8"/>
@@ -4396,7 +4374,7 @@
       <c r="J94" s="8"/>
       <c r="K94" s="8"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="95">
       <c r="A95" s="8"/>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
@@ -4409,7 +4387,7 @@
       <c r="J95" s="8"/>
       <c r="K95" s="8"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="96">
       <c r="A96" s="8"/>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
@@ -4422,7 +4400,7 @@
       <c r="J96" s="8"/>
       <c r="K96" s="8"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97">
       <c r="A97" s="8"/>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
@@ -4435,7 +4413,7 @@
       <c r="J97" s="8"/>
       <c r="K97" s="8"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="98">
       <c r="A98" s="8"/>
       <c r="B98" s="8"/>
       <c r="C98" s="8"/>
@@ -4448,7 +4426,7 @@
       <c r="J98" s="8"/>
       <c r="K98" s="8"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99">
       <c r="A99" s="8"/>
       <c r="B99" s="8"/>
       <c r="C99" s="8"/>
@@ -4461,7 +4439,7 @@
       <c r="J99" s="8"/>
       <c r="K99" s="8"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100">
       <c r="A100" s="8"/>
       <c r="B100" s="8"/>
       <c r="C100" s="8"/>
@@ -4474,7 +4452,7 @@
       <c r="J100" s="8"/>
       <c r="K100" s="8"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101">
       <c r="A101" s="8"/>
       <c r="B101" s="8"/>
       <c r="C101" s="8"/>
@@ -4487,7 +4465,7 @@
       <c r="J101" s="8"/>
       <c r="K101" s="8"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="102">
       <c r="A102" s="8"/>
       <c r="B102" s="8"/>
       <c r="C102" s="8"/>
@@ -4500,7 +4478,7 @@
       <c r="J102" s="8"/>
       <c r="K102" s="8"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="103">
       <c r="A103" s="8"/>
       <c r="B103" s="8"/>
       <c r="C103" s="8"/>
@@ -4513,7 +4491,7 @@
       <c r="J103" s="8"/>
       <c r="K103" s="8"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="104">
       <c r="A104" s="8"/>
       <c r="B104" s="8"/>
       <c r="C104" s="8"/>
@@ -4526,7 +4504,7 @@
       <c r="J104" s="8"/>
       <c r="K104" s="8"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="105">
       <c r="A105" s="8"/>
       <c r="B105" s="8"/>
       <c r="C105" s="8"/>
@@ -4539,7 +4517,7 @@
       <c r="J105" s="8"/>
       <c r="K105" s="8"/>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="106">
       <c r="A106" s="8"/>
       <c r="B106" s="8"/>
       <c r="C106" s="8"/>
@@ -4552,7 +4530,7 @@
       <c r="J106" s="8"/>
       <c r="K106" s="8"/>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107">
       <c r="A107" s="8"/>
       <c r="B107" s="8"/>
       <c r="C107" s="8"/>
@@ -4565,7 +4543,7 @@
       <c r="J107" s="8"/>
       <c r="K107" s="8"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="108">
       <c r="A108" s="8"/>
       <c r="B108" s="8"/>
       <c r="C108" s="8"/>
@@ -4578,7 +4556,7 @@
       <c r="J108" s="8"/>
       <c r="K108" s="8"/>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="109">
       <c r="A109" s="8"/>
       <c r="B109" s="8"/>
       <c r="C109" s="8"/>
@@ -4591,7 +4569,7 @@
       <c r="J109" s="8"/>
       <c r="K109" s="8"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="110">
       <c r="A110" s="8"/>
       <c r="B110" s="8"/>
       <c r="C110" s="8"/>
@@ -4604,7 +4582,7 @@
       <c r="J110" s="8"/>
       <c r="K110" s="8"/>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="111">
       <c r="A111" s="8"/>
       <c r="B111" s="8"/>
       <c r="C111" s="8"/>
@@ -4617,7 +4595,7 @@
       <c r="J111" s="8"/>
       <c r="K111" s="8"/>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="112">
       <c r="A112" s="8"/>
       <c r="B112" s="8"/>
       <c r="C112" s="8"/>
@@ -4630,7 +4608,7 @@
       <c r="J112" s="8"/>
       <c r="K112" s="8"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="113">
       <c r="A113" s="8"/>
       <c r="B113" s="8"/>
       <c r="C113" s="8"/>
@@ -4643,7 +4621,7 @@
       <c r="J113" s="8"/>
       <c r="K113" s="8"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="114">
       <c r="A114" s="8"/>
       <c r="B114" s="8"/>
       <c r="C114" s="8"/>
@@ -4656,7 +4634,7 @@
       <c r="J114" s="8"/>
       <c r="K114" s="8"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="115">
       <c r="A115" s="8"/>
       <c r="B115" s="8"/>
       <c r="C115" s="8"/>
@@ -4669,7 +4647,7 @@
       <c r="J115" s="8"/>
       <c r="K115" s="8"/>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="116">
       <c r="A116" s="8"/>
       <c r="B116" s="8"/>
       <c r="C116" s="8"/>
@@ -4682,7 +4660,7 @@
       <c r="J116" s="8"/>
       <c r="K116" s="8"/>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="117">
       <c r="A117" s="8"/>
       <c r="B117" s="8"/>
       <c r="C117" s="8"/>
@@ -4695,7 +4673,7 @@
       <c r="J117" s="8"/>
       <c r="K117" s="8"/>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="118">
       <c r="A118" s="8"/>
       <c r="B118" s="8"/>
       <c r="C118" s="8"/>
@@ -4708,7 +4686,7 @@
       <c r="J118" s="8"/>
       <c r="K118" s="8"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="119">
       <c r="A119" s="8"/>
       <c r="B119" s="8"/>
       <c r="C119" s="8"/>
@@ -4721,7 +4699,7 @@
       <c r="J119" s="8"/>
       <c r="K119" s="8"/>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="120">
       <c r="A120" s="8"/>
       <c r="B120" s="8"/>
       <c r="C120" s="8"/>
@@ -4734,7 +4712,7 @@
       <c r="J120" s="8"/>
       <c r="K120" s="8"/>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="121">
       <c r="A121" s="8"/>
       <c r="B121" s="8"/>
       <c r="C121" s="8"/>
@@ -4747,7 +4725,7 @@
       <c r="J121" s="8"/>
       <c r="K121" s="8"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="122">
       <c r="A122" s="8"/>
       <c r="B122" s="8"/>
       <c r="C122" s="8"/>
@@ -4760,7 +4738,7 @@
       <c r="J122" s="8"/>
       <c r="K122" s="8"/>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="123">
       <c r="A123" s="8"/>
       <c r="B123" s="8"/>
       <c r="C123" s="8"/>
@@ -4773,7 +4751,7 @@
       <c r="J123" s="8"/>
       <c r="K123" s="8"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="124">
       <c r="A124" s="8"/>
       <c r="B124" s="8"/>
       <c r="C124" s="8"/>
@@ -4786,7 +4764,7 @@
       <c r="J124" s="8"/>
       <c r="K124" s="8"/>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="125">
       <c r="A125" s="8"/>
       <c r="B125" s="8"/>
       <c r="C125" s="8"/>
@@ -4799,7 +4777,7 @@
       <c r="J125" s="8"/>
       <c r="K125" s="8"/>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="126">
       <c r="A126" s="8"/>
       <c r="B126" s="8"/>
       <c r="C126" s="8"/>
@@ -4812,7 +4790,7 @@
       <c r="J126" s="8"/>
       <c r="K126" s="8"/>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="127">
       <c r="A127" s="8"/>
       <c r="B127" s="8"/>
       <c r="C127" s="8"/>
@@ -4825,7 +4803,7 @@
       <c r="J127" s="8"/>
       <c r="K127" s="8"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="128">
       <c r="A128" s="8"/>
       <c r="B128" s="8"/>
       <c r="C128" s="8"/>
@@ -4838,7 +4816,7 @@
       <c r="J128" s="8"/>
       <c r="K128" s="8"/>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="129">
       <c r="A129" s="8"/>
       <c r="B129" s="8"/>
       <c r="C129" s="8"/>
@@ -4851,7 +4829,7 @@
       <c r="J129" s="8"/>
       <c r="K129" s="8"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="130">
       <c r="A130" s="8"/>
       <c r="B130" s="8"/>
       <c r="C130" s="8"/>
@@ -4864,7 +4842,7 @@
       <c r="J130" s="8"/>
       <c r="K130" s="8"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="131">
       <c r="A131" s="8"/>
       <c r="B131" s="8"/>
       <c r="C131" s="8"/>
@@ -4877,7 +4855,7 @@
       <c r="J131" s="8"/>
       <c r="K131" s="8"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="132">
       <c r="A132" s="8"/>
       <c r="B132" s="8"/>
       <c r="C132" s="8"/>
@@ -4890,7 +4868,7 @@
       <c r="J132" s="8"/>
       <c r="K132" s="8"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="133">
       <c r="A133" s="8"/>
       <c r="B133" s="8"/>
       <c r="C133" s="8"/>
@@ -4903,7 +4881,7 @@
       <c r="J133" s="8"/>
       <c r="K133" s="8"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="134">
       <c r="A134" s="8"/>
       <c r="B134" s="8"/>
       <c r="C134" s="8"/>
@@ -4916,7 +4894,7 @@
       <c r="J134" s="8"/>
       <c r="K134" s="8"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="135">
       <c r="A135" s="8"/>
       <c r="B135" s="8"/>
       <c r="C135" s="8"/>
@@ -4929,7 +4907,7 @@
       <c r="J135" s="8"/>
       <c r="K135" s="8"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="136">
       <c r="A136" s="8"/>
       <c r="B136" s="8"/>
       <c r="C136" s="8"/>
@@ -4942,7 +4920,7 @@
       <c r="J136" s="8"/>
       <c r="K136" s="8"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="137">
       <c r="A137" s="8"/>
       <c r="B137" s="8"/>
       <c r="C137" s="8"/>
@@ -4955,7 +4933,7 @@
       <c r="J137" s="8"/>
       <c r="K137" s="8"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="138">
       <c r="A138" s="8"/>
       <c r="B138" s="8"/>
       <c r="C138" s="8"/>
@@ -4968,7 +4946,7 @@
       <c r="J138" s="8"/>
       <c r="K138" s="8"/>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="139">
       <c r="A139" s="8"/>
       <c r="B139" s="8"/>
       <c r="C139" s="8"/>
@@ -4981,7 +4959,7 @@
       <c r="J139" s="8"/>
       <c r="K139" s="8"/>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="140">
       <c r="A140" s="8"/>
       <c r="B140" s="8"/>
       <c r="C140" s="8"/>
@@ -4994,7 +4972,7 @@
       <c r="J140" s="8"/>
       <c r="K140" s="8"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="141">
       <c r="A141" s="8"/>
       <c r="B141" s="8"/>
       <c r="C141" s="8"/>
@@ -5007,7 +4985,7 @@
       <c r="J141" s="8"/>
       <c r="K141" s="8"/>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="142">
       <c r="A142" s="8"/>
       <c r="B142" s="8"/>
       <c r="C142" s="8"/>
@@ -5020,7 +4998,7 @@
       <c r="J142" s="8"/>
       <c r="K142" s="8"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="143">
       <c r="A143" s="8"/>
       <c r="B143" s="8"/>
       <c r="C143" s="8"/>
@@ -5033,7 +5011,7 @@
       <c r="J143" s="8"/>
       <c r="K143" s="8"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="144">
       <c r="A144" s="8"/>
       <c r="B144" s="8"/>
       <c r="C144" s="8"/>
@@ -5046,7 +5024,7 @@
       <c r="J144" s="8"/>
       <c r="K144" s="8"/>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="145">
       <c r="A145" s="8"/>
       <c r="B145" s="8"/>
       <c r="C145" s="8"/>
@@ -5059,7 +5037,7 @@
       <c r="J145" s="8"/>
       <c r="K145" s="8"/>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="146">
       <c r="A146" s="8"/>
       <c r="B146" s="8"/>
       <c r="C146" s="8"/>
@@ -5072,7 +5050,7 @@
       <c r="J146" s="8"/>
       <c r="K146" s="8"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="147">
       <c r="A147" s="8"/>
       <c r="B147" s="8"/>
       <c r="C147" s="8"/>
@@ -5085,7 +5063,7 @@
       <c r="J147" s="8"/>
       <c r="K147" s="8"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="148">
       <c r="A148" s="8"/>
       <c r="B148" s="8"/>
       <c r="C148" s="8"/>
@@ -5098,7 +5076,7 @@
       <c r="J148" s="8"/>
       <c r="K148" s="8"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="149">
       <c r="A149" s="8"/>
       <c r="B149" s="8"/>
       <c r="C149" s="8"/>
@@ -5111,7 +5089,7 @@
       <c r="J149" s="8"/>
       <c r="K149" s="8"/>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="150">
       <c r="A150" s="8"/>
       <c r="B150" s="8"/>
       <c r="C150" s="8"/>
@@ -5124,7 +5102,7 @@
       <c r="J150" s="8"/>
       <c r="K150" s="8"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="151">
       <c r="A151" s="8"/>
       <c r="B151" s="8"/>
       <c r="C151" s="8"/>
@@ -5137,7 +5115,7 @@
       <c r="J151" s="8"/>
       <c r="K151" s="8"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="152">
       <c r="A152" s="8"/>
       <c r="B152" s="8"/>
       <c r="C152" s="8"/>
@@ -5150,7 +5128,7 @@
       <c r="J152" s="8"/>
       <c r="K152" s="8"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="153">
       <c r="A153" s="8"/>
       <c r="B153" s="8"/>
       <c r="C153" s="8"/>
@@ -5163,7 +5141,7 @@
       <c r="J153" s="8"/>
       <c r="K153" s="8"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="154">
       <c r="A154" s="8"/>
       <c r="B154" s="8"/>
       <c r="C154" s="8"/>
@@ -5176,7 +5154,7 @@
       <c r="J154" s="8"/>
       <c r="K154" s="8"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="155">
       <c r="A155" s="8"/>
       <c r="B155" s="8"/>
       <c r="C155" s="8"/>
@@ -5189,7 +5167,7 @@
       <c r="J155" s="8"/>
       <c r="K155" s="8"/>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="156">
       <c r="A156" s="8"/>
       <c r="B156" s="8"/>
       <c r="C156" s="8"/>
@@ -5202,7 +5180,7 @@
       <c r="J156" s="8"/>
       <c r="K156" s="8"/>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="157">
       <c r="A157" s="8"/>
       <c r="B157" s="8"/>
       <c r="C157" s="8"/>
@@ -5215,7 +5193,7 @@
       <c r="J157" s="8"/>
       <c r="K157" s="8"/>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="158">
       <c r="A158" s="8"/>
       <c r="B158" s="8"/>
       <c r="C158" s="8"/>
@@ -5228,7 +5206,7 @@
       <c r="J158" s="8"/>
       <c r="K158" s="8"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="159">
       <c r="A159" s="8"/>
       <c r="B159" s="8"/>
       <c r="C159" s="8"/>
@@ -5241,7 +5219,7 @@
       <c r="J159" s="8"/>
       <c r="K159" s="8"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="160">
       <c r="A160" s="8"/>
       <c r="B160" s="8"/>
       <c r="C160" s="8"/>
@@ -5254,7 +5232,7 @@
       <c r="J160" s="8"/>
       <c r="K160" s="8"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="161">
       <c r="A161" s="8"/>
       <c r="B161" s="8"/>
       <c r="C161" s="8"/>
@@ -5267,7 +5245,7 @@
       <c r="J161" s="8"/>
       <c r="K161" s="8"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="162">
       <c r="A162" s="8"/>
       <c r="B162" s="8"/>
       <c r="C162" s="8"/>
@@ -5280,7 +5258,7 @@
       <c r="J162" s="8"/>
       <c r="K162" s="8"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="163">
       <c r="A163" s="8"/>
       <c r="B163" s="8"/>
       <c r="C163" s="8"/>
@@ -5293,7 +5271,7 @@
       <c r="J163" s="8"/>
       <c r="K163" s="8"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="164">
       <c r="A164" s="8"/>
       <c r="B164" s="8"/>
       <c r="C164" s="8"/>
@@ -5306,7 +5284,7 @@
       <c r="J164" s="8"/>
       <c r="K164" s="8"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="165">
       <c r="A165" s="8"/>
       <c r="B165" s="8"/>
       <c r="C165" s="8"/>
@@ -5319,7 +5297,7 @@
       <c r="J165" s="8"/>
       <c r="K165" s="8"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="166">
       <c r="A166" s="8"/>
       <c r="B166" s="8"/>
       <c r="C166" s="8"/>
@@ -5332,7 +5310,7 @@
       <c r="J166" s="8"/>
       <c r="K166" s="8"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="167">
       <c r="A167" s="8"/>
       <c r="B167" s="8"/>
       <c r="C167" s="8"/>
@@ -5345,7 +5323,7 @@
       <c r="J167" s="8"/>
       <c r="K167" s="8"/>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="168">
       <c r="A168" s="8"/>
       <c r="B168" s="8"/>
       <c r="C168" s="8"/>
@@ -5358,7 +5336,7 @@
       <c r="J168" s="8"/>
       <c r="K168" s="8"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="169">
       <c r="A169" s="8"/>
       <c r="B169" s="8"/>
       <c r="C169" s="8"/>
@@ -5371,7 +5349,7 @@
       <c r="J169" s="8"/>
       <c r="K169" s="8"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="170">
       <c r="A170" s="8"/>
       <c r="B170" s="8"/>
       <c r="C170" s="8"/>
@@ -5384,7 +5362,7 @@
       <c r="J170" s="8"/>
       <c r="K170" s="8"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="171">
       <c r="A171" s="8"/>
       <c r="B171" s="8"/>
       <c r="C171" s="8"/>
@@ -5397,7 +5375,7 @@
       <c r="J171" s="8"/>
       <c r="K171" s="8"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="172">
       <c r="A172" s="8"/>
       <c r="B172" s="8"/>
       <c r="C172" s="8"/>
@@ -5410,7 +5388,7 @@
       <c r="J172" s="8"/>
       <c r="K172" s="8"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="173">
       <c r="A173" s="8"/>
       <c r="B173" s="8"/>
       <c r="C173" s="8"/>
@@ -5423,7 +5401,7 @@
       <c r="J173" s="8"/>
       <c r="K173" s="8"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="174">
       <c r="A174" s="8"/>
       <c r="B174" s="8"/>
       <c r="C174" s="8"/>
@@ -5436,7 +5414,7 @@
       <c r="J174" s="8"/>
       <c r="K174" s="8"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="175">
       <c r="A175" s="8"/>
       <c r="B175" s="8"/>
       <c r="C175" s="8"/>
@@ -5449,7 +5427,7 @@
       <c r="J175" s="8"/>
       <c r="K175" s="8"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="176">
       <c r="A176" s="8"/>
       <c r="B176" s="8"/>
       <c r="C176" s="8"/>
@@ -5462,7 +5440,7 @@
       <c r="J176" s="8"/>
       <c r="K176" s="8"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="177">
       <c r="A177" s="8"/>
       <c r="B177" s="8"/>
       <c r="C177" s="8"/>
@@ -5475,7 +5453,7 @@
       <c r="J177" s="8"/>
       <c r="K177" s="8"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="178">
       <c r="A178" s="8"/>
       <c r="B178" s="8"/>
       <c r="C178" s="8"/>
@@ -5488,7 +5466,7 @@
       <c r="J178" s="8"/>
       <c r="K178" s="8"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="179">
       <c r="A179" s="8"/>
       <c r="B179" s="8"/>
       <c r="C179" s="8"/>
@@ -5501,7 +5479,7 @@
       <c r="J179" s="8"/>
       <c r="K179" s="8"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="180">
       <c r="A180" s="8"/>
       <c r="B180" s="8"/>
       <c r="C180" s="8"/>
@@ -5514,7 +5492,7 @@
       <c r="J180" s="8"/>
       <c r="K180" s="8"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="181">
       <c r="A181" s="8"/>
       <c r="B181" s="8"/>
       <c r="C181" s="8"/>
@@ -5527,7 +5505,7 @@
       <c r="J181" s="8"/>
       <c r="K181" s="8"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="182">
       <c r="A182" s="8"/>
       <c r="B182" s="8"/>
       <c r="C182" s="8"/>
@@ -5540,7 +5518,7 @@
       <c r="J182" s="8"/>
       <c r="K182" s="8"/>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="183">
       <c r="A183" s="8"/>
       <c r="B183" s="8"/>
       <c r="C183" s="8"/>
@@ -5553,7 +5531,7 @@
       <c r="J183" s="8"/>
       <c r="K183" s="8"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="184">
       <c r="A184" s="8"/>
       <c r="B184" s="8"/>
       <c r="C184" s="8"/>
@@ -5566,7 +5544,7 @@
       <c r="J184" s="8"/>
       <c r="K184" s="8"/>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="185">
       <c r="A185" s="8"/>
       <c r="B185" s="8"/>
       <c r="C185" s="8"/>
@@ -5579,7 +5557,7 @@
       <c r="J185" s="8"/>
       <c r="K185" s="8"/>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="186">
       <c r="A186" s="8"/>
       <c r="B186" s="8"/>
       <c r="C186" s="8"/>
@@ -5592,7 +5570,7 @@
       <c r="J186" s="8"/>
       <c r="K186" s="8"/>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="187">
       <c r="A187" s="8"/>
       <c r="B187" s="8"/>
       <c r="C187" s="8"/>
@@ -5605,7 +5583,7 @@
       <c r="J187" s="8"/>
       <c r="K187" s="8"/>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="188">
       <c r="A188" s="8"/>
       <c r="B188" s="8"/>
       <c r="C188" s="8"/>
@@ -5618,7 +5596,7 @@
       <c r="J188" s="8"/>
       <c r="K188" s="8"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="189">
       <c r="A189" s="8"/>
       <c r="B189" s="8"/>
       <c r="C189" s="8"/>
@@ -5631,7 +5609,7 @@
       <c r="J189" s="8"/>
       <c r="K189" s="8"/>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="190">
       <c r="A190" s="8"/>
       <c r="B190" s="8"/>
       <c r="C190" s="8"/>
@@ -5644,7 +5622,7 @@
       <c r="J190" s="8"/>
       <c r="K190" s="8"/>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="191">
       <c r="A191" s="8"/>
       <c r="B191" s="8"/>
       <c r="C191" s="8"/>
@@ -5657,7 +5635,7 @@
       <c r="J191" s="8"/>
       <c r="K191" s="8"/>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="192">
       <c r="A192" s="8"/>
       <c r="B192" s="8"/>
       <c r="C192" s="8"/>
@@ -5670,7 +5648,7 @@
       <c r="J192" s="8"/>
       <c r="K192" s="8"/>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="193">
       <c r="A193" s="8"/>
       <c r="B193" s="8"/>
       <c r="C193" s="8"/>
@@ -5683,7 +5661,7 @@
       <c r="J193" s="8"/>
       <c r="K193" s="8"/>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="194">
       <c r="A194" s="8"/>
       <c r="B194" s="8"/>
       <c r="C194" s="8"/>
@@ -5696,7 +5674,7 @@
       <c r="J194" s="8"/>
       <c r="K194" s="8"/>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="195">
       <c r="A195" s="8"/>
       <c r="B195" s="8"/>
       <c r="C195" s="8"/>
@@ -5709,7 +5687,7 @@
       <c r="J195" s="8"/>
       <c r="K195" s="8"/>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="196">
       <c r="A196" s="8"/>
       <c r="B196" s="8"/>
       <c r="C196" s="8"/>
@@ -5722,7 +5700,7 @@
       <c r="J196" s="8"/>
       <c r="K196" s="8"/>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="197">
       <c r="A197" s="8"/>
       <c r="B197" s="8"/>
       <c r="C197" s="8"/>
@@ -5735,7 +5713,7 @@
       <c r="J197" s="8"/>
       <c r="K197" s="8"/>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="198">
       <c r="A198" s="8"/>
       <c r="B198" s="8"/>
       <c r="C198" s="8"/>
@@ -5748,7 +5726,7 @@
       <c r="J198" s="8"/>
       <c r="K198" s="8"/>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="199">
       <c r="A199" s="8"/>
       <c r="B199" s="8"/>
       <c r="C199" s="8"/>
@@ -5761,7 +5739,7 @@
       <c r="J199" s="8"/>
       <c r="K199" s="8"/>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="200">
       <c r="A200" s="8"/>
       <c r="B200" s="8"/>
       <c r="C200" s="8"/>
@@ -5774,7 +5752,7 @@
       <c r="J200" s="8"/>
       <c r="K200" s="8"/>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="201">
       <c r="A201" s="8"/>
       <c r="B201" s="8"/>
       <c r="C201" s="8"/>
@@ -5787,7 +5765,7 @@
       <c r="J201" s="8"/>
       <c r="K201" s="8"/>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="202">
       <c r="A202" s="8"/>
       <c r="B202" s="8"/>
       <c r="C202" s="8"/>
@@ -5800,7 +5778,7 @@
       <c r="J202" s="8"/>
       <c r="K202" s="8"/>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="203">
       <c r="A203" s="8"/>
       <c r="B203" s="8"/>
       <c r="C203" s="8"/>
@@ -5813,7 +5791,7 @@
       <c r="J203" s="8"/>
       <c r="K203" s="8"/>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="204">
       <c r="A204" s="8"/>
       <c r="B204" s="8"/>
       <c r="C204" s="8"/>
@@ -5826,7 +5804,7 @@
       <c r="J204" s="8"/>
       <c r="K204" s="8"/>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="205">
       <c r="A205" s="8"/>
       <c r="B205" s="8"/>
       <c r="C205" s="8"/>
@@ -5839,7 +5817,7 @@
       <c r="J205" s="8"/>
       <c r="K205" s="8"/>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="206">
       <c r="A206" s="8"/>
       <c r="B206" s="8"/>
       <c r="C206" s="8"/>
@@ -5852,7 +5830,7 @@
       <c r="J206" s="8"/>
       <c r="K206" s="8"/>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="207">
       <c r="A207" s="8"/>
       <c r="B207" s="8"/>
       <c r="C207" s="8"/>
@@ -5865,7 +5843,7 @@
       <c r="J207" s="8"/>
       <c r="K207" s="8"/>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="208">
       <c r="A208" s="8"/>
       <c r="B208" s="8"/>
       <c r="C208" s="8"/>
@@ -5878,7 +5856,7 @@
       <c r="J208" s="8"/>
       <c r="K208" s="8"/>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="209">
       <c r="A209" s="8"/>
       <c r="B209" s="8"/>
       <c r="C209" s="8"/>
@@ -5891,7 +5869,7 @@
       <c r="J209" s="8"/>
       <c r="K209" s="8"/>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="210">
       <c r="A210" s="8"/>
       <c r="B210" s="8"/>
       <c r="C210" s="8"/>
@@ -5904,7 +5882,7 @@
       <c r="J210" s="8"/>
       <c r="K210" s="8"/>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="211">
       <c r="A211" s="8"/>
       <c r="B211" s="8"/>
       <c r="C211" s="8"/>
@@ -5917,7 +5895,7 @@
       <c r="J211" s="8"/>
       <c r="K211" s="8"/>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="212">
       <c r="A212" s="8"/>
       <c r="B212" s="8"/>
       <c r="C212" s="8"/>
@@ -5930,7 +5908,7 @@
       <c r="J212" s="8"/>
       <c r="K212" s="8"/>
     </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="213">
       <c r="A213" s="8"/>
       <c r="B213" s="8"/>
       <c r="C213" s="8"/>
@@ -5943,7 +5921,7 @@
       <c r="J213" s="8"/>
       <c r="K213" s="8"/>
     </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="214">
       <c r="A214" s="8"/>
       <c r="B214" s="8"/>
       <c r="C214" s="8"/>
@@ -5956,7 +5934,7 @@
       <c r="J214" s="8"/>
       <c r="K214" s="8"/>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="215">
       <c r="A215" s="8"/>
       <c r="B215" s="8"/>
       <c r="C215" s="8"/>
@@ -5969,7 +5947,7 @@
       <c r="J215" s="8"/>
       <c r="K215" s="8"/>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="216">
       <c r="A216" s="8"/>
       <c r="B216" s="8"/>
       <c r="C216" s="8"/>
@@ -5982,7 +5960,7 @@
       <c r="J216" s="8"/>
       <c r="K216" s="8"/>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="217">
       <c r="A217" s="8"/>
       <c r="B217" s="8"/>
       <c r="C217" s="8"/>
@@ -5995,7 +5973,7 @@
       <c r="J217" s="8"/>
       <c r="K217" s="8"/>
     </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="218">
       <c r="A218" s="8"/>
       <c r="B218" s="8"/>
       <c r="C218" s="8"/>
@@ -6008,7 +5986,7 @@
       <c r="J218" s="8"/>
       <c r="K218" s="8"/>
     </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="219">
       <c r="A219" s="8"/>
       <c r="B219" s="8"/>
       <c r="C219" s="8"/>
@@ -6021,7 +5999,7 @@
       <c r="J219" s="8"/>
       <c r="K219" s="8"/>
     </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="220">
       <c r="A220" s="8"/>
       <c r="B220" s="8"/>
       <c r="C220" s="8"/>
@@ -6034,7 +6012,7 @@
       <c r="J220" s="8"/>
       <c r="K220" s="8"/>
     </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="221">
       <c r="A221" s="8"/>
       <c r="B221" s="8"/>
       <c r="C221" s="8"/>
@@ -6070,44 +6048,45 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" customWidth="1"/>
-    <col min="5" max="6" width="25.6640625" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" customWidth="1"/>
-    <col min="8" max="8" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-    </row>
-    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
         <v>173</v>
       </c>
@@ -6133,7 +6112,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="45" customHeight="1">
       <c r="A4" s="10" t="s">
         <v>180</v>
       </c>
@@ -6159,59 +6138,59 @@
         <v>187</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5">
+      <c r="A5" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="E5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="14" t="s">
+      <c r="G5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="18" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+    <row r="6">
+      <c r="A6" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="14" t="s">
+      <c r="G6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="18" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -6221,7 +6200,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -6231,7 +6210,7 @@
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -6241,7 +6220,7 @@
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -6251,7 +6230,7 @@
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -6261,7 +6240,7 @@
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -6271,7 +6250,7 @@
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -6281,7 +6260,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -6291,7 +6270,7 @@
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -6301,7 +6280,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -6311,7 +6290,7 @@
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -6321,7 +6300,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -6331,7 +6310,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -6341,7 +6320,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -6351,7 +6330,7 @@
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -6361,7 +6340,7 @@
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -6371,7 +6350,7 @@
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -6381,7 +6360,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -6391,7 +6370,7 @@
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -6401,7 +6380,7 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -6430,36 +6409,36 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-    </row>
-    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>64</v>
       </c>
@@ -6476,7 +6455,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="11" t="s">
         <v>231</v>
       </c>
@@ -6493,7 +6472,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" ht="50" customHeight="1">
       <c r="A6" s="11" t="s">
         <v>90</v>
       </c>
@@ -6510,7 +6489,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>100</v>
       </c>
@@ -6527,7 +6506,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" ht="50" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>95</v>
       </c>
@@ -6544,7 +6523,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>105</v>
       </c>
@@ -6561,7 +6540,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" ht="50" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>110</v>
       </c>
@@ -6578,7 +6557,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>117</v>
       </c>
@@ -6595,7 +6574,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" ht="50" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>121</v>
       </c>
@@ -6610,6 +6589,23 @@
       </c>
       <c r="E12" s="11" t="s">
         <v>230</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>234</v>
+      </c>
+      <c r="B13" t="s">
+        <v>235</v>
+      </c>
+      <c r="C13" t="s">
+        <v>236</v>
+      </c>
+      <c r="D13" t="s">
+        <v>237</v>
+      </c>
+      <c r="E13" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>